<commit_message>
Presentacion de los cinco tableros, todas las ITS y Chile frente al mundo
PowerPoint interactivo con indice, antes y ahora, metricas, hallazgos, medidas y conclusiones. Tablero ITS con pagina Todas las ITS (10 infecciones) y comparacion con EE.UU. y Europa. README con iconos y miniaturas.
</commit_message>
<xml_diff>
--- a/dashboard-its-chile/ITS_Chile_BaseDatos.xlsx
+++ b/dashboard-its-chile/ITS_Chile_BaseDatos.xlsx
@@ -30,7 +30,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SimCondon" sheetId="21" state="visible" r:id="rId21"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SimIndicadores" sheetId="22" state="visible" r:id="rId22"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SimSupuestos" sheetId="23" state="visible" r:id="rId23"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TodasITS" sheetId="24" state="visible" r:id="rId24"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ChileMundoITS" sheetId="25" state="visible" r:id="rId25"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Fuentes" sheetId="26" state="visible" r:id="rId26"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -367,7 +369,39 @@
 </file>
 
 <file path=xl/tables/table23.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="Fuentes" displayName="Fuentes" ref="A1:C40" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="23" name="TodasITS" displayName="TodasITS" ref="A1:G11" headerRowCount="1">
+  <autoFilter ref="A1:G11"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="Orden"/>
+    <tableColumn id="2" name="ITS"/>
+    <tableColumn id="3" name="Chile"/>
+    <tableColumn id="4" name="Vigilancia"/>
+    <tableColumn id="5" name="Mundo"/>
+    <tableColumn id="6" name="QueEs"/>
+    <tableColumn id="7" name="FuenteID"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table24.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="24" name="ChileMundoITS" displayName="ChileMundoITS" ref="A1:G10" headerRowCount="1">
+  <autoFilter ref="A1:G10"/>
+  <tableColumns count="7">
+    <tableColumn id="1" name="ITS"/>
+    <tableColumn id="2" name="OrdenITS"/>
+    <tableColumn id="3" name="Lugar"/>
+    <tableColumn id="4" name="OrdenLugar"/>
+    <tableColumn id="5" name="Tasa"/>
+    <tableColumn id="6" name="Anio"/>
+    <tableColumn id="7" name="FuenteID"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleLight1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table25.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="25" name="Fuentes" displayName="Fuentes" ref="A1:C54" headerRowCount="1">
   <autoFilter ref="A1:C35"/>
   <tableColumns count="3">
     <tableColumn id="1" name="FuenteID"/>
@@ -785,7 +819,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -7357,7 +7390,762 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C40"/>
+  <dimension ref="A1:G11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="46" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="44" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Orden</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>ITS</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Vigilancia</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Mundo</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>QueEs</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>FuenteID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Sífilis</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>11.155 casos · 55,2 por 100 mil (2025)</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>Notificación obligatoria</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>8 millones de casos nuevos al año (2022)</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>Bacteria · se cura con penicilina</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>S2;S21;S47</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Gonorrea</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>2.682 casos · 13,3 por 100 mil (2025)</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Notificación obligatoria</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>82 millones de casos nuevos al año (2020)</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>Bacteria · se cura con antibiótico</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>S4;S27;S47</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>VIH</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>4.313 diagnósticos (2025) · 91.000 viven con VIH</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>Notificación obligatoria</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>41 millones viven con VIH; 1,2 millones de infecciones nuevas (2025)</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>Virus · tratamiento de por vida; indetectable = intransmisible</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>S10;S12;S46;S47</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Hepatitis B</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>609 casos (2021) · 2 de cada 3 por vía sexual</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Notificación obligatoria</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>254 millones viven con hepatitis B (2022)</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>Virus · se previene con vacuna</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>S25;S54;S47</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Mpox</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>1.455 confirmados (jun 2022 – jun 2024)</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Solo laboratorio o estudios</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Más de 180 mil casos y 492 muertes (2022 – mar 2026)</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>Virus · notificación inmediata como evento emergente</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>S56;S55</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Clamidia</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Sin tasa nacional · 5,9% en embarazadas de Santiago (estudio 2010–11)</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Solo laboratorio o estudios</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>129 millones de casos nuevos al año (2020)</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>Bacteria · se cura con antibiótico; suele no dar síntomas</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>S48;S49;S47</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>VPH (virus papiloma)</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>17,1% en mujeres en tamizaje (estudio 2014–2023)</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Solo laboratorio o estudios</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>1 de cada 3 hombres tiene VPH genital</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>Virus · se previene con vacuna; causa cáncer cervicouterino</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>S50;S51</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Herpes genital</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Sin dato poblacional</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>No se vigila</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>520 millones viven con herpes tipo 2</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>Virus · no se cura; los brotes se tratan</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>S52</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Tricomoniasis</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>2,4% en embarazadas de Santiago (estudio 2010–11)</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>No se vigila</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>156 millones de casos nuevos al año (2020)</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>Parásito · se cura con antibiótico</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>S48;S53</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Linfogranuloma venéreo</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Sin dato público</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>No se vigila</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Europa: 3.490 casos (2024)</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>Bacteria (clamidia L1–L3) · se cura con antibiótico</t>
+        </is>
+      </c>
+      <c r="G11" s="3" t="inlineStr">
+        <is>
+          <t>S57</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet25.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G10"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="9" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ITS</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>OrdenITS</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Lugar</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>OrdenLugar</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Tasa</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>Anio</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>FuenteID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Sífilis</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>S2</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Sífilis</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>EE.UU.</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>62.5</v>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>S44</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Sífilis</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>10.8</v>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="inlineStr">
+        <is>
+          <t>S16</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>VIH (diagnósticos)</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>2025 (cálculo propio)</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="inlineStr">
+        <is>
+          <t>S10</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>VIH (diagnósticos)</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>EE.UU.</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr">
+        <is>
+          <t>S45</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>VIH (diagnósticos)</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>5.3</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>S18</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Gonorrea</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Chile</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>13.3</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr">
+        <is>
+          <t>S4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Gonorrea</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>EE.UU.</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>179.5</v>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>S44</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Gonorrea</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Unión Europea</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
+        <is>
+          <t>S17</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet26.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -8042,6 +8830,244 @@
       <c r="C40" t="inlineStr">
         <is>
           <t>https://www.who.int/news-room/questions-and-answers/item/comprehensive-sexuality-education</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>S44</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>CDC, Sexually Transmitted Infections Surveillance 2023 (tasas de sífilis, gonorrea y clamidia en EE.UU.).</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.cdc.gov/sti-statistics/annual/index.html</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>S45</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>CDC, HIV Surveillance Report: diagnósticos de VIH 2023 en EE.UU.</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>https://stacks.cdc.gov/view/cdc/177771</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>S46</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>ONUSIDA, ficha mundial 2026 (datos 2025).</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>https://www.unaids.org/sites/default/files/2026-06/20260612_Global_HIV_Factsheet.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>S47</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Decreto 7/2019 MINSAL: reglamento de enfermedades de notificación obligatoria.</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>https://www.diariooficial.interior.gob.cl/publicaciones/2020/01/24/42561/01/1715587.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>S48</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Rev Chil Infectol 2012: Chlamydia trachomatis y Trichomonas vaginalis en embarazadas de Santiago.</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>https://pesquisa.bvsalud.org/gim/resource/en/lil-660024</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>S49</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>OMS, nota descriptiva: clamidia.</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news-room/fact-sheets/detail/chlamydia</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>S50</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Rev Méd Chile 2026: prevalencia de VPH en mujeres en tamizaje (Huechuraba 2014–2023).</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>https://www.revistamedicadechile.cl/</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>S51</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>OMS 2023: uno de cada tres hombres en el mundo tiene VPH genital.</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news/item/01-09-2023-one-in-three-men-worldwide-are-infected-with-genital-human-papillomavirus</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>S52</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>OMS 2024: más de 1 de cada 5 adultos en el mundo tiene herpes genital.</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news/item/11-12-2024-over-1-in-5-adults-worldwide-has-a-genital-herpes-infection-who</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>S53</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>OMS, nota descriptiva: tricomoniasis.</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>https://www.who.int/news-room/fact-sheets/detail/Trichomoniasis</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>S54</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>OPS/OMS 2024: hepatitis virales en el mundo (Informe mundial de hepatitis 2024).</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>https://www.paho.org/en/news/10-4-2024-who-sounds-alarm-viral-hepatitis-infections-claiming-3500-lives-each-day</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>S55</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>OPS, actualización epidemiológica de mpox (abril 2026).</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.paho.org/sites/default/files/2026/04/23042026actualizacion-epi-mpoxesfinal.pdf</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>S56</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>MINSAL, casos de mpox en Chile 2022–2024 (vía El Dínamo, 14-08-2024).</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>https://www.eldinamo.cl/sociedad/2024/08/14/oms-declara-emergencia-sanitaria-internacional-por-viruela-del-mono-cuantos-casos-hay-en-chile-y-como-se-contagia/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>S57</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>ECDC, linfogranuloma venéreo, informe anual 2024.</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>https://www.ecdc.europa.eu/en/publications-data/lymphogranuloma-venereum-annual-epidemiological-report-2024</t>
         </is>
       </c>
     </row>

</xml_diff>